<commit_message>
feat: update coin cell assembly, bioyond cell workstation, and resource configs
</commit_message>
<xml_diff>
--- a/unilabos/devices/workstation/bioyond_studio/bioyond_cell/20260323-1.xlsx
+++ b/unilabos/devices/workstation/bioyond_studio/bioyond_cell/20260323-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UniLabdev\Uni-Lab-OS\unilabos\devices\workstation\bioyond_studio\bioyond_cell\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A04DC97A-13C9-4EF6-9C81-CDA6C95820DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099ED6F8-7E11-4291-AA78-E518ABC1308B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2850" yWindow="2850" windowWidth="17280" windowHeight="9982" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="场景1 完成扣电and电导配液，以及部分单独软包配液" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
   <si>
     <t>算法批次</t>
   </si>
@@ -92,14 +92,6 @@
   </si>
   <si>
     <t>DP2026040204</t>
-  </si>
-  <si>
-    <t>LiFSI(g)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>EMC(g)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>DP2026040203</t>
@@ -108,6 +100,16 @@
   <si>
     <t>TEST-6</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>FEC(g)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>DP2026040205</t>
+  </si>
+  <si>
+    <t>DP2026040206</t>
   </si>
 </sst>
 </file>
@@ -516,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="8.796875" customWidth="1"/>
@@ -528,10 +530,10 @@
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="17.33203125" customWidth="1"/>
     <col min="9" max="9" width="17.19921875" customWidth="1"/>
-    <col min="10" max="11" width="9" style="9"/>
+    <col min="10" max="10" width="9" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -560,18 +562,15 @@
         <v>8</v>
       </c>
       <c r="J1" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="K1" s="13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="C2" s="6">
         <v>46104</v>
@@ -580,10 +579,10 @@
         <v>9</v>
       </c>
       <c r="E2" s="4">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F2" s="7">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="G2" s="4">
         <v>0</v>
@@ -595,15 +594,12 @@
         <v>0</v>
       </c>
       <c r="J2" s="14">
-        <v>0.25</v>
-      </c>
-      <c r="K2" s="14">
         <v>4.6500000000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>10</v>
@@ -615,10 +611,10 @@
         <v>9</v>
       </c>
       <c r="E3" s="4">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F3" s="7">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="G3" s="4">
         <v>0</v>
@@ -630,39 +626,74 @@
         <v>0</v>
       </c>
       <c r="J3" s="14">
-        <v>0.19</v>
-      </c>
-      <c r="K3" s="14">
         <v>4.3600000000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-    </row>
-    <row r="5" spans="1:11" ht="15" x14ac:dyDescent="0.4">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-    </row>
-    <row r="6" spans="1:11" ht="15" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10" ht="15" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="6">
+        <v>46104</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="4">
+        <v>30</v>
+      </c>
+      <c r="F4" s="7">
+        <v>2</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="14">
+        <v>4.3330000000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="6">
+        <v>46104</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="4">
+        <v>30</v>
+      </c>
+      <c r="F5" s="7">
+        <v>2</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="14">
+        <v>4.79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15" x14ac:dyDescent="0.4">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="6"/>
@@ -673,9 +704,8 @@
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-    </row>
-    <row r="7" spans="1:11" ht="15" x14ac:dyDescent="0.4">
+    </row>
+    <row r="7" spans="1:10" ht="15" x14ac:dyDescent="0.4">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="6"/>
@@ -686,9 +716,8 @@
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="3"/>
@@ -699,9 +728,8 @@
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="3"/>
@@ -712,9 +740,8 @@
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="3"/>
@@ -725,9 +752,8 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="3"/>
@@ -738,9 +764,8 @@
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="3"/>
@@ -751,9 +776,8 @@
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="3"/>
@@ -764,9 +788,8 @@
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
       <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="3"/>
@@ -777,9 +800,8 @@
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
       <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="3"/>
@@ -790,7 +812,6 @@
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>